<commit_message>
Corrida | SFE-NTTA | 2026-05-29 10:05:33.468153
</commit_message>
<xml_diff>
--- a/indicadores/SFE-NTTA_out.xlsx
+++ b/indicadores/SFE-NTTA_out.xlsx
@@ -38,7 +38,7 @@
     <t xml:space="preserve">Fuente</t>
   </si>
   <si>
-    <t xml:space="preserve">SIPA en base a ARCA y EPH INDEC</t>
+    <t xml:space="preserve">ARCA en base a SIPA y Ministerio de Economía de la provincia de Santa Fe</t>
   </si>
   <si>
     <t xml:space="preserve">Método</t>
@@ -98,7 +98,7 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">27/05/2026</t>
+    <t xml:space="preserve">29/05/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
@@ -2147,7 +2147,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.595999958907048</v>
+        <v>0.595533775810286</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2205,7 +2205,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.355215951017202</v>
+        <v>0.354660478130857</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2275,7 +2275,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.0000000279145777438761</v>
+        <v>0.0000000179049534331685</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2305,7 +2305,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.0000000459982080879348</v>
+        <v>0.000000063108839905549</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -26942,7 +26942,7 @@
         <v>514</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.00640140973530348</v>
+        <v>0.00612048126138506</v>
       </c>
     </row>
     <row r="6">
@@ -26950,7 +26950,7 @@
         <v>515</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.0368829649591526</v>
+        <v>0.03544250951204</v>
       </c>
     </row>
     <row r="7">
@@ -26958,7 +26958,7 @@
         <v>516</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0803990728762055</v>
+        <v>0.0781550150806992</v>
       </c>
     </row>
     <row r="8">
@@ -26966,7 +26966,7 @@
         <v>517</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.152954549685072</v>
+        <v>0.150824072474046</v>
       </c>
     </row>
     <row r="9">
@@ -26974,7 +26974,7 @@
         <v>518</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.149527918814516</v>
+        <v>0.1468761493508</v>
       </c>
     </row>
     <row r="10">
@@ -26982,7 +26982,7 @@
         <v>519</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.210154614329456</v>
+        <v>0.208066179871754</v>
       </c>
     </row>
     <row r="11">
@@ -26990,7 +26990,7 @@
         <v>520</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.276257028140719</v>
+        <v>0.275645968232477</v>
       </c>
     </row>
     <row r="12">
@@ -26998,7 +26998,7 @@
         <v>521</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.338084117327372</v>
+        <v>0.336596272914338</v>
       </c>
     </row>
     <row r="13">
@@ -27006,7 +27006,7 @@
         <v>522</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.358087190461309</v>
+        <v>0.356751504510178</v>
       </c>
     </row>
     <row r="14">
@@ -27014,7 +27014,7 @@
         <v>523</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.595999958907048</v>
+        <v>0.595533775810286</v>
       </c>
     </row>
     <row r="15">
@@ -27022,7 +27022,7 @@
         <v>524</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.425414777734258</v>
+        <v>0.425160127789727</v>
       </c>
     </row>
     <row r="16">
@@ -27030,7 +27030,7 @@
         <v>525</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.490942401056213</v>
+        <v>0.490391570804615</v>
       </c>
     </row>
     <row r="17">
@@ -27038,7 +27038,7 @@
         <v>526</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.46399656351752</v>
+        <v>0.463217452845618</v>
       </c>
     </row>
     <row r="18">
@@ -27046,7 +27046,7 @@
         <v>527</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.451710699739768</v>
+        <v>0.451301267622173</v>
       </c>
     </row>
     <row r="19">
@@ -27054,7 +27054,7 @@
         <v>528</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.412966805730047</v>
+        <v>0.413330518281709</v>
       </c>
     </row>
     <row r="20">
@@ -27062,7 +27062,7 @@
         <v>529</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.44789431515362</v>
+        <v>0.448709942405159</v>
       </c>
     </row>
     <row r="21">
@@ -27070,7 +27070,7 @@
         <v>530</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.378271897603572</v>
+        <v>0.379515743645704</v>
       </c>
     </row>
     <row r="22">
@@ -27078,7 +27078,7 @@
         <v>531</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.328089324379691</v>
+        <v>0.328901559718182</v>
       </c>
     </row>
     <row r="23">
@@ -27086,7 +27086,7 @@
         <v>532</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.304068467977342</v>
+        <v>0.304572185120071</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Corrida | SFE-NTTA | 2026-06-17 11:37:10.951999
</commit_message>
<xml_diff>
--- a/indicadores/SFE-NTTA_out.xlsx
+++ b/indicadores/SFE-NTTA_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="533">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="535">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Total de empleados registrados en la provincia de Santa Fe</t>
+    <t xml:space="preserve">Total de empleados registrados</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -65,6 +65,12 @@
     <t xml:space="preserve">Regresores</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincia de Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -98,13 +104,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">29/05/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2115,9 +2121,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>17</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -2128,7 +2138,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -2142,7 +2152,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
@@ -2158,7 +2168,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -2186,7 +2196,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -2200,7 +2210,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
@@ -2228,7 +2238,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -2242,7 +2252,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -2256,7 +2266,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2270,7 +2280,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
@@ -2286,7 +2296,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2300,7 +2310,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
@@ -2448,10 +2458,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B32" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2464,10 +2474,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B33" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2491,66 +2501,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="I1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="L1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="M1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="N1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="O1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="P1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="Q1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="R1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="S1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>369.207986597209</v>
@@ -2603,7 +2613,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>371.521749686477</v>
@@ -2660,7 +2670,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>369.401738012001</v>
@@ -2717,7 +2727,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>373.794850752021</v>
@@ -2774,7 +2784,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>374.962700707325</v>
@@ -2831,7 +2841,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>377.220820809657</v>
@@ -2888,7 +2898,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>373.605467913734</v>
@@ -2945,7 +2955,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>373.854709432734</v>
@@ -3002,7 +3012,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>380.669833308548</v>
@@ -3059,7 +3069,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>384.234950135517</v>
@@ -3116,7 +3126,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>381.250603550815</v>
@@ -3173,7 +3183,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>380.361398492924</v>
@@ -3230,7 +3240,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>398.655669050447</v>
@@ -3289,7 +3299,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>369.139006576623</v>
@@ -3348,7 +3358,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>366.88381430611</v>
@@ -3407,7 +3417,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>365.166684237535</v>
@@ -3466,7 +3476,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>367.13591204496</v>
@@ -3525,7 +3535,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>368.246245839209</v>
@@ -3584,7 +3594,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>359.671298538822</v>
@@ -3643,7 +3653,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>358.997127945386</v>
@@ -3702,7 +3712,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>357.262779883787</v>
@@ -3761,7 +3771,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>346.141782126095</v>
@@ -3820,7 +3830,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>352.719809995626</v>
@@ -3879,7 +3889,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>350.572730568759</v>
@@ -3938,7 +3948,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>352.670207512396</v>
@@ -3997,7 +4007,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>359.544539762748</v>
@@ -4056,7 +4066,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>355.125081902983</v>
@@ -4115,7 +4125,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>362.511969761506</v>
@@ -4174,7 +4184,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>364.987693238408</v>
@@ -4233,7 +4243,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>365.58839564629</v>
@@ -4292,7 +4302,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>361.834772856493</v>
@@ -4351,7 +4361,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>369.857748297207</v>
@@ -4410,7 +4420,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>370.038023771903</v>
@@ -4469,7 +4479,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>372.69235038977</v>
@@ -4528,7 +4538,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>375.266748184699</v>
@@ -4587,7 +4597,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>381.93561754897</v>
@@ -4646,7 +4656,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>381.232461597409</v>
@@ -4705,7 +4715,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>384.359420936848</v>
@@ -4764,7 +4774,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>384.515599725235</v>
@@ -4823,7 +4833,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>384.461967642839</v>
@@ -4882,7 +4892,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>387.266248517035</v>
@@ -4941,7 +4951,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>392.712044573776</v>
@@ -5000,7 +5010,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>382.536298868594</v>
@@ -5059,7 +5069,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>387.646755213505</v>
@@ -5118,7 +5128,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>386.143738746163</v>
@@ -5177,7 +5187,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>388.72106699815</v>
@@ -5236,7 +5246,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>391.588518322412</v>
@@ -5295,7 +5305,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>394.291862349971</v>
@@ -5354,7 +5364,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>393.052660005585</v>
@@ -5413,7 +5423,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>396.539445639685</v>
@@ -5472,7 +5482,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>399.072398087899</v>
@@ -5531,7 +5541,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>401.110114661401</v>
@@ -5590,7 +5600,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>402.099876732746</v>
@@ -5649,7 +5659,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>394.623386266837</v>
@@ -5708,7 +5718,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>390.054987513788</v>
@@ -5767,7 +5777,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>387.83989579384</v>
@@ -5826,7 +5836,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>392.575899898107</v>
@@ -5885,7 +5895,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>395.339181110073</v>
@@ -5944,7 +5954,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>397.851111290763</v>
@@ -6003,7 +6013,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>401.19503065017</v>
@@ -6062,7 +6072,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>399.546006662406</v>
@@ -6121,7 +6131,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>429.439099432951</v>
@@ -6180,7 +6190,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>430.49523533228</v>
@@ -6239,7 +6249,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>429.485377353699</v>
@@ -6298,7 +6308,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>420.582221298288</v>
@@ -6357,7 +6367,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>425.329231282782</v>
@@ -6416,7 +6426,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>428.477522855023</v>
@@ -6475,7 +6485,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>424.187565173658</v>
@@ -6534,7 +6544,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>425.247266780969</v>
@@ -6593,7 +6603,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>423.911527203472</v>
@@ -6652,7 +6662,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>425.026823643231</v>
@@ -6711,7 +6721,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>427.679614256932</v>
@@ -6770,7 +6780,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>438.212846008021</v>
@@ -6829,7 +6839,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>439.622304780518</v>
@@ -6888,7 +6898,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>438.012319138395</v>
@@ -6947,7 +6957,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>441.919099589638</v>
@@ -7006,7 +7016,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>441.222526406935</v>
@@ -7065,7 +7075,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>440.701009463213</v>
@@ -7124,7 +7134,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>441.18769795649</v>
@@ -7183,7 +7193,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>437.694058764899</v>
@@ -7242,7 +7252,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>436.965490716115</v>
@@ -7301,7 +7311,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>440.792927481009</v>
@@ -7360,7 +7370,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>442.763779200229</v>
@@ -7419,7 +7429,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>446.425972921617</v>
@@ -7478,7 +7488,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>453.007283006572</v>
@@ -7537,7 +7547,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>452.629431581031</v>
@@ -7596,7 +7606,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>449.051454077486</v>
@@ -7655,7 +7665,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>450.394810263169</v>
@@ -7714,7 +7724,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>450.777044717595</v>
@@ -7773,7 +7783,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>447.80013202491</v>
@@ -7832,7 +7842,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>449.344232164099</v>
@@ -7891,7 +7901,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>448.130768792959</v>
@@ -7950,7 +7960,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>445.831462355926</v>
@@ -8009,7 +8019,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>439.749582799641</v>
@@ -8068,7 +8078,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>442.236263982143</v>
@@ -8127,7 +8137,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>442.436102244744</v>
@@ -8186,7 +8196,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>440.679916358476</v>
@@ -8245,7 +8255,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>429.474239209735</v>
@@ -8304,7 +8314,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>426.319838031758</v>
@@ -8363,7 +8373,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>427.288741378011</v>
@@ -8422,7 +8432,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>427.980424772944</v>
@@ -8481,7 +8491,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>425.494857598861</v>
@@ -8540,7 +8550,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>423.667449121141</v>
@@ -8599,7 +8609,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>421.388974057292</v>
@@ -8658,7 +8668,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>420.616839773015</v>
@@ -8717,7 +8727,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>423.623493887664</v>
@@ -8776,7 +8786,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>427.528594432517</v>
@@ -8835,7 +8845,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>426.890421739687</v>
@@ -8894,7 +8904,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>432.14670931448</v>
@@ -8953,7 +8963,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>423.87960201907</v>
@@ -9012,7 +9022,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>424.575655246918</v>
@@ -9071,7 +9081,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>430.77659507169</v>
@@ -9130,7 +9140,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>433.780982307192</v>
@@ -9189,7 +9199,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>433.293902352127</v>
@@ -9248,7 +9258,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>439.305048339029</v>
@@ -9307,7 +9317,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>437.258641769304</v>
@@ -9366,7 +9376,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>440.765693843534</v>
@@ -9425,7 +9435,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>447.463703607938</v>
@@ -9484,7 +9494,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>448.795123688587</v>
@@ -9543,7 +9553,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>455.257984071164</v>
@@ -9602,7 +9612,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>461.956318922443</v>
@@ -9661,7 +9671,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>460.26948543253</v>
@@ -9720,7 +9730,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>462.010615972054</v>
@@ -9779,7 +9789,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>471.075716535329</v>
@@ -9838,7 +9848,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>474.391962738144</v>
@@ -9897,7 +9907,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>478.073460195595</v>
@@ -9956,7 +9966,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>479.246101335271</v>
@@ -10015,7 +10025,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>484.955458252673</v>
@@ -10074,7 +10084,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>485.981727726797</v>
@@ -10133,7 +10143,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>489.29126829239</v>
@@ -10192,7 +10202,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>495.685449038985</v>
@@ -10251,7 +10261,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>503.020901404464</v>
@@ -10310,7 +10320,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>510.430557740285</v>
@@ -10369,7 +10379,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>504.835681252123</v>
@@ -10428,7 +10438,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>504.640732400214</v>
@@ -10487,7 +10497,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>513.486690901524</v>
@@ -10546,7 +10556,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>516.018150655389</v>
@@ -10605,7 +10615,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>517.681383698973</v>
@@ -10664,7 +10674,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>516.96251153112</v>
@@ -10723,7 +10733,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>519.125783169371</v>
@@ -10782,7 +10792,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>524.830476875832</v>
@@ -10841,7 +10851,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>530.353252356919</v>
@@ -10900,7 +10910,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>536.132622790108</v>
@@ -10959,7 +10969,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>542.477698706565</v>
@@ -11018,7 +11028,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>551.688745190574</v>
@@ -11077,7 +11087,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>546.386422992099</v>
@@ -11136,7 +11146,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>543.208803558335</v>
@@ -11195,7 +11205,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>551.272016962352</v>
@@ -11254,7 +11264,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>552.40007108191</v>
@@ -11313,7 +11323,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>553.555393499415</v>
@@ -11372,7 +11382,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>557.567488204345</v>
@@ -11431,7 +11441,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>555.883461595122</v>
@@ -11490,7 +11500,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>558.161999986713</v>
@@ -11549,7 +11559,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>562.590588482464</v>
@@ -11608,7 +11618,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>567.292807132847</v>
@@ -11667,7 +11677,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>572.616776843523</v>
@@ -11726,7 +11736,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>580.397788286682</v>
@@ -11785,7 +11795,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>574.63584960018</v>
@@ -11844,7 +11854,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>573.310771349317</v>
@@ -11903,7 +11913,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>572.435362426339</v>
@@ -11962,7 +11972,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>583.444636463757</v>
@@ -12021,7 +12031,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>582.424290996005</v>
@@ -12080,7 +12090,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>586.760686311199</v>
@@ -12139,7 +12149,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>588.201289278075</v>
@@ -12198,7 +12208,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>590.957958436188</v>
@@ -12257,7 +12267,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>600.553305261559</v>
@@ -12316,7 +12326,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>601.119470533897</v>
@@ -12375,7 +12385,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>605.609163441711</v>
@@ -12434,7 +12444,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>613.791911337325</v>
@@ -12493,7 +12503,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>602.86288670668</v>
@@ -12552,7 +12562,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>603.151573469949</v>
@@ -12611,7 +12621,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>610.7752</v>
@@ -12670,7 +12680,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>613.089933333333</v>
@@ -12729,7 +12739,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>609.354566666667</v>
@@ -12788,7 +12798,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>618.578</v>
@@ -12847,7 +12857,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>619.374</v>
@@ -12906,7 +12916,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>621.653</v>
@@ -12965,7 +12975,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>623.934</v>
@@ -13024,7 +13034,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>627.839</v>
@@ -13083,7 +13093,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>625.609</v>
@@ -13142,7 +13152,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>627.246033333333</v>
@@ -13201,7 +13211,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>614.2633</v>
@@ -13260,7 +13270,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>609.7233</v>
@@ -13319,7 +13329,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>611.969033333333</v>
@@ -13378,7 +13388,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>609.703033333333</v>
@@ -13437,7 +13447,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>607.480666666667</v>
@@ -13496,7 +13506,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>607.378033333333</v>
@@ -13555,7 +13565,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>605.724666666667</v>
@@ -13614,7 +13624,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>604.756266666667</v>
@@ -13673,7 +13683,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>611.839866666667</v>
@@ -13732,7 +13742,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>614.531666666667</v>
@@ -13791,7 +13801,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>615.635833333333</v>
@@ -13850,7 +13860,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>619.820633333333</v>
@@ -13909,7 +13919,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>610.084633333333</v>
@@ -13968,7 +13978,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>611.096133333333</v>
@@ -14027,7 +14037,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>619.0033</v>
@@ -14086,7 +14096,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>620.373366666667</v>
@@ -14145,7 +14155,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>619.610066666667</v>
@@ -14204,7 +14214,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>620.783133333333</v>
@@ -14263,7 +14273,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>622.004033333333</v>
@@ -14322,7 +14332,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>624.737633333333</v>
@@ -14381,7 +14391,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>626.6403</v>
@@ -14440,7 +14450,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>630.9673</v>
@@ -14499,7 +14509,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>637.968766666667</v>
@@ -14558,7 +14568,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>645.6607</v>
@@ -14617,7 +14627,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>639.453133333333</v>
@@ -14676,7 +14686,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>639.018533333333</v>
@@ -14735,7 +14745,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>644.560466666667</v>
@@ -14794,7 +14804,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>648.540133333333</v>
@@ -14853,7 +14863,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>650.994866666667</v>
@@ -14912,7 +14922,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>653.1129</v>
@@ -14971,7 +14981,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>652.459933333333</v>
@@ -15030,7 +15040,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>657.748733333333</v>
@@ -15089,7 +15099,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>657.937666666667</v>
@@ -15148,7 +15158,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>660.345966666667</v>
@@ -15207,7 +15217,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>665.8099</v>
@@ -15266,7 +15276,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>669.251266666667</v>
@@ -15325,7 +15335,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>661.341366666667</v>
@@ -15384,7 +15394,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>659.163266666667</v>
@@ -15443,7 +15453,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>665.2767</v>
@@ -15502,7 +15512,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>666.4771</v>
@@ -15561,7 +15571,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>665.999266666667</v>
@@ -15620,7 +15630,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>665.2558</v>
@@ -15679,7 +15689,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>663.733</v>
@@ -15738,7 +15748,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>663.881</v>
@@ -15797,7 +15807,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>664.215</v>
@@ -15856,7 +15866,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>669.365</v>
@@ -15915,7 +15925,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>669.328</v>
@@ -15974,7 +15984,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>672.003</v>
@@ -16033,7 +16043,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>667.846</v>
@@ -16092,7 +16102,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>665.408</v>
@@ -16151,7 +16161,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>673.7</v>
@@ -16210,7 +16220,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>679.447</v>
@@ -16269,7 +16279,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>680.047</v>
@@ -16328,7 +16338,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>676.854</v>
@@ -16387,7 +16397,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>678.69</v>
@@ -16446,7 +16456,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>681.002</v>
@@ -16505,7 +16515,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>680.902</v>
@@ -16564,7 +16574,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>684.054</v>
@@ -16623,7 +16633,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>687.655</v>
@@ -16682,7 +16692,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>688.59</v>
@@ -16741,7 +16751,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>684.239</v>
@@ -16800,7 +16810,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>678.834</v>
@@ -16859,7 +16869,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>679.244</v>
@@ -16918,7 +16928,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>682.881</v>
@@ -16977,7 +16987,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>682.961</v>
@@ -17036,7 +17046,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>684.696</v>
@@ -17095,7 +17105,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>684.401</v>
@@ -17154,7 +17164,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>685.173</v>
@@ -17213,7 +17223,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>685.982</v>
@@ -17272,7 +17282,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>690.37</v>
@@ -17331,7 +17341,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>692.79</v>
@@ -17390,7 +17400,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>693.019</v>
@@ -17449,7 +17459,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>688.924</v>
@@ -17508,7 +17518,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>688.028</v>
@@ -17567,7 +17577,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>695.41</v>
@@ -17626,7 +17636,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>700.992</v>
@@ -17685,7 +17695,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>701.57</v>
@@ -17744,7 +17754,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>706.255</v>
@@ -17803,7 +17813,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>703.984</v>
@@ -17862,7 +17872,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>706.891</v>
@@ -17921,7 +17931,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>705.626</v>
@@ -17980,7 +17990,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>710.219</v>
@@ -18039,7 +18049,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>710.635</v>
@@ -18098,7 +18108,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>707.586</v>
@@ -18157,7 +18167,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>701.133</v>
@@ -18216,7 +18226,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>700.812</v>
@@ -18275,7 +18285,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B269" s="2" t="n">
         <v>705.441</v>
@@ -18334,7 +18344,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B270" s="2" t="n">
         <v>703.954</v>
@@ -18393,7 +18403,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B271" s="2" t="n">
         <v>703.824</v>
@@ -18452,7 +18462,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B272" s="2" t="n">
         <v>703.87</v>
@@ -18511,7 +18521,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B273" s="2" t="n">
         <v>699.316</v>
@@ -18570,7 +18580,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B274" s="2" t="n">
         <v>702.962</v>
@@ -18629,7 +18639,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B275" s="2" t="n">
         <v>704.216</v>
@@ -18688,7 +18698,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B276" s="2" t="n">
         <v>706.538</v>
@@ -18747,7 +18757,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B277" s="2" t="n">
         <v>710.009</v>
@@ -18806,7 +18816,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B278" s="2" t="n">
         <v>711.448</v>
@@ -18865,7 +18875,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B279" s="2" t="n">
         <v>705.579</v>
@@ -18924,7 +18934,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B280" s="2" t="n">
         <v>706.422</v>
@@ -18983,7 +18993,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B281" s="2" t="n">
         <v>711.903</v>
@@ -19042,7 +19052,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B282" s="2" t="n">
         <v>709.014</v>
@@ -19101,7 +19111,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B283" s="2" t="n">
         <v>713.672</v>
@@ -19160,7 +19170,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B284" s="2" t="n">
         <v>711.713</v>
@@ -19219,7 +19229,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B285" s="2" t="n">
         <v>709.289</v>
@@ -19278,7 +19288,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B286" s="2" t="n">
         <v>715.506</v>
@@ -19337,7 +19347,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B287" s="2" t="n">
         <v>714.532</v>
@@ -19396,7 +19406,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B288" s="2" t="n">
         <v>722.187</v>
@@ -19455,7 +19465,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B289" s="2" t="n">
         <v>722.353</v>
@@ -19514,7 +19524,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B290" s="2" t="n">
         <v>721.084</v>
@@ -19573,7 +19583,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B291" s="2" t="n">
         <v>713.475</v>
@@ -19632,7 +19642,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B292" s="2" t="n">
         <v>712.037</v>
@@ -19691,7 +19701,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B293" s="2" t="n">
         <v>716.132</v>
@@ -19750,7 +19760,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B294" s="2" t="n">
         <v>714.59</v>
@@ -19809,7 +19819,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B295" s="2" t="n">
         <v>717.065</v>
@@ -19868,7 +19878,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B296" s="2" t="n">
         <v>712.994</v>
@@ -19927,7 +19937,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B297" s="2" t="n">
         <v>710.87</v>
@@ -19986,7 +19996,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B298" s="2" t="n">
         <v>716.267</v>
@@ -20045,7 +20055,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B299" s="2" t="n">
         <v>713.642</v>
@@ -20104,7 +20114,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B300" s="2" t="n">
         <v>715.067</v>
@@ -20163,7 +20173,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B301" s="2" t="n">
         <v>711.87</v>
@@ -20222,7 +20232,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B302" s="2" t="n">
         <v>710.224</v>
@@ -20281,7 +20291,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B303" s="2" t="n">
         <v>703.373</v>
@@ -20340,7 +20350,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B304" s="2" t="n">
         <v>704.943</v>
@@ -20399,7 +20409,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B305" s="2" t="n">
         <v>704.873</v>
@@ -20458,7 +20468,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B306" s="2" t="n">
         <v>708.807</v>
@@ -20517,7 +20527,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B307" s="2" t="n">
         <v>706.148</v>
@@ -20576,7 +20586,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B308" s="2" t="n">
         <v>707.613</v>
@@ -20635,7 +20645,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B309" s="2" t="n">
         <v>705.816</v>
@@ -20694,7 +20704,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B310" s="2" t="n">
         <v>711.615</v>
@@ -20753,7 +20763,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B311" s="2" t="n">
         <v>705.645</v>
@@ -20812,7 +20822,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B312" s="2" t="n">
         <v>708.3615</v>
@@ -20871,7 +20881,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B313" s="2" t="n">
         <v>703.885</v>
@@ -20930,7 +20940,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B314" s="2" t="n">
         <v>699.305</v>
@@ -20989,7 +20999,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B315" s="2" t="n">
         <v>694.027</v>
@@ -21048,7 +21058,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B316" s="2" t="n">
         <v>691.16</v>
@@ -21107,7 +21117,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B317" s="2" t="n">
         <v>688.917</v>
@@ -21166,7 +21176,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B318" s="2" t="n">
         <v>680.316</v>
@@ -21225,7 +21235,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B319" s="2" t="n">
         <v>679.356</v>
@@ -21284,7 +21294,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B320" s="2" t="n">
         <v>679.3</v>
@@ -21343,7 +21353,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B321" s="2" t="n">
         <v>680.734</v>
@@ -21402,7 +21412,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B322" s="2" t="n">
         <v>680.226</v>
@@ -21461,7 +21471,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B323" s="2" t="n">
         <v>681.372</v>
@@ -21520,7 +21530,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B324" s="2" t="n">
         <v>684.843</v>
@@ -21579,7 +21589,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B325" s="2" t="n">
         <v>686.675</v>
@@ -21638,7 +21648,7 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B326" s="2" t="n">
         <v>688.072</v>
@@ -21697,7 +21707,7 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B327" s="2" t="n">
         <v>688.107</v>
@@ -21756,7 +21766,7 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B328" s="2" t="n">
         <v>690.686</v>
@@ -21815,7 +21825,7 @@
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B329" s="2" t="n">
         <v>696.709</v>
@@ -21874,7 +21884,7 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B330" s="2" t="n">
         <v>699.409</v>
@@ -21933,7 +21943,7 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B331" s="2" t="n">
         <v>697.71</v>
@@ -21992,7 +22002,7 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B332" s="2" t="n">
         <v>696.563</v>
@@ -22051,7 +22061,7 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B333" s="2" t="n">
         <v>697.243</v>
@@ -22110,7 +22120,7 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B334" s="2" t="n">
         <v>700.867</v>
@@ -22169,7 +22179,7 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B335" s="2" t="n">
         <v>705.685</v>
@@ -22228,7 +22238,7 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B336" s="2" t="n">
         <v>703.342</v>
@@ -22287,7 +22297,7 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B337" s="2" t="n">
         <v>713.201</v>
@@ -22346,7 +22356,7 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B338" s="2" t="n">
         <v>709.97</v>
@@ -22405,7 +22415,7 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B339" s="2" t="n">
         <v>704.446</v>
@@ -22464,7 +22474,7 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B340" s="2" t="n">
         <v>704.468</v>
@@ -22523,7 +22533,7 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B341" s="2" t="n">
         <v>712.555</v>
@@ -22582,7 +22592,7 @@
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B342" s="2" t="n">
         <v>714.544</v>
@@ -22641,7 +22651,7 @@
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B343" s="2" t="n">
         <v>715.23</v>
@@ -22700,7 +22710,7 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B344" s="2" t="n">
         <v>717.351</v>
@@ -22759,7 +22769,7 @@
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B345" s="2" t="n">
         <v>720.506</v>
@@ -22818,7 +22828,7 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B346" s="2" t="n">
         <v>721.402</v>
@@ -22877,7 +22887,7 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B347" s="2" t="n">
         <v>724.196</v>
@@ -22936,7 +22946,7 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B348" s="2" t="n">
         <v>727.608</v>
@@ -22995,7 +23005,7 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B349" s="2" t="n">
         <v>730.707</v>
@@ -23054,7 +23064,7 @@
     </row>
     <row r="350">
       <c r="A350" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B350" s="2" t="n">
         <v>728.61</v>
@@ -23113,7 +23123,7 @@
     </row>
     <row r="351">
       <c r="A351" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B351" s="2" t="n">
         <v>727.421</v>
@@ -23172,7 +23182,7 @@
     </row>
     <row r="352">
       <c r="A352" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B352" s="2" t="n">
         <v>727.513</v>
@@ -23231,7 +23241,7 @@
     </row>
     <row r="353">
       <c r="A353" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B353" s="2" t="n">
         <v>735.285</v>
@@ -23290,7 +23300,7 @@
     </row>
     <row r="354">
       <c r="A354" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B354" s="2" t="n">
         <v>736.948</v>
@@ -23349,7 +23359,7 @@
     </row>
     <row r="355">
       <c r="A355" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B355" s="2" t="n">
         <v>738.002</v>
@@ -23408,7 +23418,7 @@
     </row>
     <row r="356">
       <c r="A356" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B356" s="2" t="n">
         <v>741.025</v>
@@ -23467,7 +23477,7 @@
     </row>
     <row r="357">
       <c r="A357" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B357" s="2" t="n">
         <v>745.025</v>
@@ -23526,7 +23536,7 @@
     </row>
     <row r="358">
       <c r="A358" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B358" s="2" t="n">
         <v>750.841</v>
@@ -23585,7 +23595,7 @@
     </row>
     <row r="359">
       <c r="A359" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B359" s="2" t="n">
         <v>752.038</v>
@@ -23644,7 +23654,7 @@
     </row>
     <row r="360">
       <c r="A360" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B360" s="2" t="n">
         <v>753.482</v>
@@ -23703,7 +23713,7 @@
     </row>
     <row r="361">
       <c r="A361" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B361" s="2" t="n">
         <v>754.072</v>
@@ -23762,7 +23772,7 @@
     </row>
     <row r="362">
       <c r="A362" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B362" s="2" t="n">
         <v>749.687</v>
@@ -23821,7 +23831,7 @@
     </row>
     <row r="363">
       <c r="A363" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B363" s="2" t="n">
         <v>741.451</v>
@@ -23880,7 +23890,7 @@
     </row>
     <row r="364">
       <c r="A364" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B364" s="2" t="n">
         <v>738.036</v>
@@ -23939,7 +23949,7 @@
     </row>
     <row r="365">
       <c r="A365" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B365" s="2" t="n">
         <v>738.793</v>
@@ -23998,7 +24008,7 @@
     </row>
     <row r="366">
       <c r="A366" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B366" s="2" t="n">
         <v>737.625</v>
@@ -24057,7 +24067,7 @@
     </row>
     <row r="367">
       <c r="A367" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B367" s="2" t="n">
         <v>734.671</v>
@@ -24116,7 +24126,7 @@
     </row>
     <row r="368">
       <c r="A368" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B368" s="2" t="n">
         <v>731.995</v>
@@ -24175,7 +24185,7 @@
     </row>
     <row r="369">
       <c r="A369" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B369" s="2" t="n">
         <v>731.332</v>
@@ -24234,7 +24244,7 @@
     </row>
     <row r="370">
       <c r="A370" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B370" s="2" t="n">
         <v>732.934</v>
@@ -24293,7 +24303,7 @@
     </row>
     <row r="371">
       <c r="A371" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B371" s="2" t="n">
         <v>734.312</v>
@@ -24352,7 +24362,7 @@
     </row>
     <row r="372">
       <c r="A372" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B372" s="2" t="n">
         <v>737.89</v>
@@ -24411,7 +24421,7 @@
     </row>
     <row r="373">
       <c r="A373" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B373" s="2" t="n">
         <v>739.247533333333</v>
@@ -24470,7 +24480,7 @@
     </row>
     <row r="374">
       <c r="A374" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B374" s="2" t="n">
         <v>736.82</v>
@@ -24529,7 +24539,7 @@
     </row>
     <row r="375">
       <c r="A375" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B375" s="2" t="n">
         <v>731.347</v>
@@ -24588,7 +24598,7 @@
     </row>
     <row r="376">
       <c r="A376" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B376" s="2" t="n">
         <v>730.838</v>
@@ -24647,7 +24657,7 @@
     </row>
     <row r="377">
       <c r="A377" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B377" s="2" t="n">
         <v>734.537</v>
@@ -24706,7 +24716,7 @@
     </row>
     <row r="378">
       <c r="A378" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B378" s="2" t="n">
         <v>739.09</v>
@@ -24765,7 +24775,7 @@
     </row>
     <row r="379">
       <c r="A379" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B379" s="2" t="n">
         <v>737.658</v>
@@ -24824,7 +24834,7 @@
     </row>
     <row r="380">
       <c r="A380" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B380" s="2" t="n">
         <v>739.277</v>
@@ -24883,7 +24893,7 @@
     </row>
     <row r="381">
       <c r="A381" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B381" s="2" t="n">
         <v>735.953</v>
@@ -24942,7 +24952,7 @@
     </row>
     <row r="382">
       <c r="A382" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B382" s="2" t="n">
         <v>736.24</v>
@@ -25001,7 +25011,7 @@
     </row>
     <row r="383">
       <c r="A383" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B383" s="2" t="n">
         <v>737.722</v>
@@ -25060,7 +25070,7 @@
     </row>
     <row r="384">
       <c r="A384" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B384" s="2" t="n">
         <v>741.474</v>
@@ -25119,7 +25129,7 @@
     </row>
     <row r="385">
       <c r="A385" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B385" s="2" t="n">
         <v>738.858766666667</v>
@@ -25178,7 +25188,7 @@
     </row>
     <row r="386">
       <c r="A386" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B386" s="2" t="n">
         <v>738.800518643082</v>
@@ -25237,7 +25247,7 @@
     </row>
     <row r="387">
       <c r="A387" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B387" s="2" t="n">
         <v>733.80238461733</v>
@@ -25296,7 +25306,7 @@
     </row>
     <row r="388">
       <c r="A388" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B388" s="2" t="n">
         <v>733.465817731481</v>
@@ -25355,7 +25365,7 @@
     </row>
     <row r="389">
       <c r="A389" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B389" s="2" t="n">
         <v>737.723793570828</v>
@@ -25414,7 +25424,7 @@
     </row>
     <row r="390">
       <c r="A390" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B390" s="2"/>
       <c r="C390" s="3" t="n">
@@ -25445,7 +25455,7 @@
     </row>
     <row r="391">
       <c r="A391" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B391" s="2"/>
       <c r="C391" s="3" t="n">
@@ -25476,7 +25486,7 @@
     </row>
     <row r="392">
       <c r="A392" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B392" s="2"/>
       <c r="C392" s="3" t="n">
@@ -25507,7 +25517,7 @@
     </row>
     <row r="393">
       <c r="A393" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B393" s="2"/>
       <c r="C393" s="3" t="n">
@@ -25538,7 +25548,7 @@
     </row>
     <row r="394">
       <c r="A394" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B394" s="2"/>
       <c r="C394" s="3" t="n">
@@ -25569,7 +25579,7 @@
     </row>
     <row r="395">
       <c r="A395" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B395" s="2"/>
       <c r="C395" s="3" t="n">
@@ -25600,7 +25610,7 @@
     </row>
     <row r="396">
       <c r="A396" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B396" s="2"/>
       <c r="C396" s="3" t="n">
@@ -25631,7 +25641,7 @@
     </row>
     <row r="397">
       <c r="A397" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B397" s="2"/>
       <c r="C397" s="3" t="n">
@@ -25662,7 +25672,7 @@
     </row>
     <row r="398">
       <c r="A398" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B398" s="2"/>
       <c r="C398" s="3" t="n">
@@ -25693,7 +25703,7 @@
     </row>
     <row r="399">
       <c r="A399" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B399" s="2"/>
       <c r="C399" s="3" t="n">
@@ -25724,7 +25734,7 @@
     </row>
     <row r="400">
       <c r="A400" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B400" s="2"/>
       <c r="C400" s="3" t="n">
@@ -25755,7 +25765,7 @@
     </row>
     <row r="401">
       <c r="A401" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B401" s="2"/>
       <c r="C401" s="3" t="n">
@@ -25786,7 +25796,7 @@
     </row>
     <row r="402">
       <c r="A402" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B402" s="2"/>
       <c r="C402" s="3"/>
@@ -25809,7 +25819,7 @@
     </row>
     <row r="403">
       <c r="A403" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B403" s="2"/>
       <c r="C403" s="3"/>
@@ -25832,7 +25842,7 @@
     </row>
     <row r="404">
       <c r="A404" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B404" s="2"/>
       <c r="C404" s="3"/>
@@ -25855,7 +25865,7 @@
     </row>
     <row r="405">
       <c r="A405" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B405" s="2"/>
       <c r="C405" s="3"/>
@@ -25878,7 +25888,7 @@
     </row>
     <row r="406">
       <c r="A406" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B406" s="2"/>
       <c r="C406" s="3"/>
@@ -25901,7 +25911,7 @@
     </row>
     <row r="407">
       <c r="A407" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B407" s="2"/>
       <c r="C407" s="3"/>
@@ -25924,7 +25934,7 @@
     </row>
     <row r="408">
       <c r="A408" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B408" s="2"/>
       <c r="C408" s="3"/>
@@ -25947,7 +25957,7 @@
     </row>
     <row r="409">
       <c r="A409" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B409" s="2"/>
       <c r="C409" s="3"/>
@@ -25970,7 +25980,7 @@
     </row>
     <row r="410">
       <c r="A410" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B410" s="2"/>
       <c r="C410" s="3"/>
@@ -25993,7 +26003,7 @@
     </row>
     <row r="411">
       <c r="A411" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B411" s="2"/>
       <c r="C411" s="3"/>
@@ -26016,7 +26026,7 @@
     </row>
     <row r="412">
       <c r="A412" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B412" s="2"/>
       <c r="C412" s="3"/>
@@ -26039,7 +26049,7 @@
     </row>
     <row r="413">
       <c r="A413" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B413" s="2"/>
       <c r="C413" s="3"/>
@@ -26062,7 +26072,7 @@
     </row>
     <row r="414">
       <c r="A414" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B414" s="2"/>
       <c r="C414" s="3"/>
@@ -26085,7 +26095,7 @@
     </row>
     <row r="415">
       <c r="A415" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B415" s="2"/>
       <c r="C415" s="3"/>
@@ -26108,7 +26118,7 @@
     </row>
     <row r="416">
       <c r="A416" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B416" s="2"/>
       <c r="C416" s="3"/>
@@ -26131,7 +26141,7 @@
     </row>
     <row r="417">
       <c r="A417" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B417" s="2"/>
       <c r="C417" s="3"/>
@@ -26154,7 +26164,7 @@
     </row>
     <row r="418">
       <c r="A418" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B418" s="2"/>
       <c r="C418" s="3"/>
@@ -26177,7 +26187,7 @@
     </row>
     <row r="419">
       <c r="A419" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B419" s="2"/>
       <c r="C419" s="3"/>
@@ -26200,7 +26210,7 @@
     </row>
     <row r="420">
       <c r="A420" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B420" s="2"/>
       <c r="C420" s="3"/>
@@ -26223,7 +26233,7 @@
     </row>
     <row r="421">
       <c r="A421" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B421" s="2"/>
       <c r="C421" s="3"/>
@@ -26246,7 +26256,7 @@
     </row>
     <row r="422">
       <c r="A422" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B422" s="2"/>
       <c r="C422" s="3"/>
@@ -26269,7 +26279,7 @@
     </row>
     <row r="423">
       <c r="A423" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B423" s="2"/>
       <c r="C423" s="3"/>
@@ -26292,7 +26302,7 @@
     </row>
     <row r="424">
       <c r="A424" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B424" s="2"/>
       <c r="C424" s="3"/>
@@ -26315,7 +26325,7 @@
     </row>
     <row r="425">
       <c r="A425" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B425" s="2"/>
       <c r="C425" s="3"/>
@@ -26338,7 +26348,7 @@
     </row>
     <row r="426">
       <c r="A426" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B426" s="2"/>
       <c r="C426" s="3"/>
@@ -26361,7 +26371,7 @@
     </row>
     <row r="427">
       <c r="A427" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B427" s="2"/>
       <c r="C427" s="3"/>
@@ -26384,7 +26394,7 @@
     </row>
     <row r="428">
       <c r="A428" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B428" s="2"/>
       <c r="C428" s="3"/>
@@ -26407,7 +26417,7 @@
     </row>
     <row r="429">
       <c r="A429" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B429" s="2"/>
       <c r="C429" s="3"/>
@@ -26430,7 +26440,7 @@
     </row>
     <row r="430">
       <c r="A430" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B430" s="2"/>
       <c r="C430" s="3"/>
@@ -26453,7 +26463,7 @@
     </row>
     <row r="431">
       <c r="A431" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B431" s="2"/>
       <c r="C431" s="3"/>
@@ -26476,7 +26486,7 @@
     </row>
     <row r="432">
       <c r="A432" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B432" s="2"/>
       <c r="C432" s="3"/>
@@ -26499,7 +26509,7 @@
     </row>
     <row r="433">
       <c r="A433" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B433" s="2"/>
       <c r="C433" s="3"/>
@@ -26522,7 +26532,7 @@
     </row>
     <row r="434">
       <c r="A434" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B434" s="2"/>
       <c r="C434" s="3"/>
@@ -26545,7 +26555,7 @@
     </row>
     <row r="435">
       <c r="A435" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B435" s="2"/>
       <c r="C435" s="3"/>
@@ -26568,7 +26578,7 @@
     </row>
     <row r="436">
       <c r="A436" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B436" s="2"/>
       <c r="C436" s="3"/>
@@ -26591,7 +26601,7 @@
     </row>
     <row r="437">
       <c r="A437" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="B437" s="2"/>
       <c r="C437" s="3"/>
@@ -26614,7 +26624,7 @@
     </row>
     <row r="438">
       <c r="A438" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B438" s="2"/>
       <c r="C438" s="3"/>
@@ -26637,7 +26647,7 @@
     </row>
     <row r="439">
       <c r="A439" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B439" s="2"/>
       <c r="C439" s="3"/>
@@ -26660,7 +26670,7 @@
     </row>
     <row r="440">
       <c r="A440" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B440" s="2"/>
       <c r="C440" s="3"/>
@@ -26683,7 +26693,7 @@
     </row>
     <row r="441">
       <c r="A441" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B441" s="2"/>
       <c r="C441" s="3"/>
@@ -26706,7 +26716,7 @@
     </row>
     <row r="442">
       <c r="A442" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B442" s="2"/>
       <c r="C442" s="3"/>
@@ -26729,7 +26739,7 @@
     </row>
     <row r="443">
       <c r="A443" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B443" s="2"/>
       <c r="C443" s="3"/>
@@ -26752,7 +26762,7 @@
     </row>
     <row r="444">
       <c r="A444" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B444" s="2"/>
       <c r="C444" s="3"/>
@@ -26775,7 +26785,7 @@
     </row>
     <row r="445">
       <c r="A445" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B445" s="2"/>
       <c r="C445" s="3"/>
@@ -26809,97 +26819,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
   </sheetData>
@@ -26923,7 +26933,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -26933,13 +26943,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>0.00612048126138506</v>
@@ -26947,7 +26957,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>0.03544250951204</v>
@@ -26955,7 +26965,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>0.0781550150806992</v>
@@ -26963,7 +26973,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0.150824072474046</v>
@@ -26971,7 +26981,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0.1468761493508</v>
@@ -26979,7 +26989,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0.208066179871754</v>
@@ -26987,7 +26997,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0.275645968232477</v>
@@ -26995,7 +27005,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0.336596272914338</v>
@@ -27003,7 +27013,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>0.356751504510178</v>
@@ -27011,7 +27021,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>0.595533775810286</v>
@@ -27019,7 +27029,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>0.425160127789727</v>
@@ -27027,7 +27037,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>0.490391570804615</v>
@@ -27035,7 +27045,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>0.463217452845618</v>
@@ -27043,7 +27053,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>0.451301267622173</v>
@@ -27051,7 +27061,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>0.413330518281709</v>
@@ -27059,7 +27069,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>0.448709942405159</v>
@@ -27067,7 +27077,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>0.379515743645704</v>
@@ -27075,7 +27085,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>0.328901559718182</v>
@@ -27083,7 +27093,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>0.304572185120071</v>

</xml_diff>